<commit_message>
chore: update feature audit tracker after verification
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Ra27231f3a8654063"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R469cdd0cb7f74a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Ra072877e49b94d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R59ac7b3abd124bd2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1467,19 +1467,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I27" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J27" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K27" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L27" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M27" s="10" t="str">
-        <x:v>Failure paths are defined but not unit-tested.</x:v>
+        <x:v>Verified in an end-to-end run on 2026-07-01 with the README sample YouTube URL; failure paths are still not unit-tested.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1687,7 +1687,7 @@
         <x:v>Times, speed, and local-model markers are zeroed in the manual subtitle result; README now matches the narrower condition that this path only applies when diarization is inactive and `--local` is not set.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="33" ht="66" hidden="0" customHeight="1">
       <x:c r="A33" s="11" t="str">
         <x:v>FT-REMOTE-09</x:v>
       </x:c>
@@ -1713,19 +1713,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I33" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J33" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L33" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M33" s="10" t="str">
-        <x:v>Remote alias smoke tests cover `-l/--local/--prefer-local-for-remote` but not download failure paths.</x:v>
+        <x:v>Remote alias smoke tests cover the forced-local flags, and a full run on 2026-07-01 against the README sample YouTube URL completed with `transcript_source = downloaded-audio-local-model`.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="66" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
fix: reject ambiguous spaced flag values
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Ra072877e49b94d90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R59ac7b3abd124bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R88813e0216484751"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd12f975c19c042f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -621,7 +621,7 @@
         <x:v>Prevents accidental creation of files like `-Z`.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="7" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A7" s="11" t="str">
         <x:v>FT-CLI-06</x:v>
       </x:c>
@@ -647,19 +647,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I7" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J7" s="12" t="str">
-        <x:v>Parser edge case</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K7" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L7" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M7" s="10" t="str">
-        <x:v>Space-separated invalid optional values can fall through as positional args instead of erroring immediately.</x:v>
+        <x:v>Verified by new unit and CLI smoke tests: invalid spaced values after `--speakers` or `--text` now error instead of becoming positional output paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -908,7 +908,7 @@
         <x:v>Ordinary repetition and longer words are intentionally left alone.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="14" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A14" s="11" t="str">
         <x:v>FT-CLI-13</x:v>
       </x:c>
@@ -934,19 +934,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I14" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J14" s="12" t="str">
-        <x:v>Parser edge case</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K14" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L14" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M14" s="10" t="str">
-        <x:v>`--diarize none` is rejected in favor of `-D`; invalid spaced values after bare `--diarize` can be reinterpreted positionally.</x:v>
+        <x:v>`--diarize none` is still rejected in favor of `-D`, and invalid spaced values after bare `--diarize` now error instead of being reinterpreted as positional output paths.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
fix: reject flag tokens as missing option values
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R88813e0216484751"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd12f975c19c042f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R262814a44ee3429c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re889945150624707"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -498,7 +498,7 @@
         <x:v>Automated tests passed and the README now states that speaker-aware text is the default on-disk output.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="4" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
         <x:v>FT-CLI-03</x:v>
       </x:c>
@@ -524,19 +524,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I4" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J4" s="12" t="str">
-        <x:v>None logged</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K4" s="12" t="str">
-        <x:v>Not needed</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L4" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M4" s="10" t="str">
-        <x:v>Existing directories receive the default filename inside them.</x:v>
+        <x:v>Smoke coverage already proved normal destination modes, and the parser now rejects `--output` followed by another flag instead of writing to a file literally named after that flag.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -949,7 +949,7 @@
         <x:v>`--diarize none` is still rejected in favor of `-D`, and invalid spaced values after bare `--diarize` now error instead of being reinterpreted as positional output paths.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="15" ht="66" hidden="0" customHeight="1">
       <x:c r="A15" s="11" t="str">
         <x:v>FT-CLI-14</x:v>
       </x:c>
@@ -975,19 +975,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I15" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J15" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K15" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L15" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M15" s="10" t="str">
-        <x:v>Happy-path smoke coverage exists; most rejection cases are unit-only or untested.</x:v>
+        <x:v>Happy-path smoke coverage already exercised chunk/model/remote overrides, and new unit+smoke tests now prove that `--model-dir`, `--model-package`, and `--model-url` reject a following flag token as a missing value.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh feature audit tracker
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R262814a44ee3429c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Re889945150624707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Ra58635771d374f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R35032fff9d914cfd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -442,7 +442,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I2" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J2" s="12" t="str">
         <x:v>None logged</x:v>
@@ -451,7 +451,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L2" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M2" s="10" t="str">
         <x:v>Short-circuit precedence over invalid trailing args is code-defined but not explicitly smoke-tested.</x:v>
@@ -565,7 +565,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I5" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J5" s="12" t="str">
         <x:v>None logged</x:v>
@@ -574,7 +574,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L5" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M5" s="10" t="str">
         <x:v>Messages vary slightly by path but enforce the same contract.</x:v>
@@ -606,7 +606,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I6" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J6" s="12" t="str">
         <x:v>None logged</x:v>
@@ -615,7 +615,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L6" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M6" s="10" t="str">
         <x:v>Prevents accidental creation of files like `-Z`.</x:v>
@@ -688,7 +688,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I8" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
         <x:v>Edge behavior only</x:v>
@@ -697,7 +697,7 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M8" s="10" t="str">
         <x:v>If `segments` is absent, speaker output renders as an empty string.</x:v>
@@ -729,7 +729,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I9" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
         <x:v>Missing-segment gap</x:v>
@@ -738,7 +738,7 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M9" s="10" t="str">
         <x:v>Timestamped text with no segments renders empty output.</x:v>
@@ -770,7 +770,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I10" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J10" s="12" t="str">
         <x:v>None logged</x:v>
@@ -779,7 +779,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L10" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M10" s="10" t="str">
         <x:v>Missing-helper warnings are intentionally suppressed in text mode.</x:v>
@@ -893,7 +893,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I13" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J13" s="12" t="str">
         <x:v>None logged</x:v>
@@ -902,7 +902,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L13" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M13" s="10" t="str">
         <x:v>Ordinary repetition and longer words are intentionally left alone.</x:v>
@@ -1180,7 +1180,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I20" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J20" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1189,7 +1189,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L20" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M20" s="10" t="str">
         <x:v>Sample rounding can shift exact chunk boundaries slightly.</x:v>
@@ -1303,7 +1303,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I23" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J23" s="12" t="str">
         <x:v>Overlap with CLI feature</x:v>
@@ -1312,7 +1312,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L23" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M23" s="10" t="str">
         <x:v>Kept as pipeline behavior because it changes the post-ASR data shape.</x:v>
@@ -1385,7 +1385,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I25" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J25" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1394,7 +1394,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L25" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M25" s="10" t="str">
         <x:v>Non-HTTP remote schemes are not supported.</x:v>
@@ -1508,7 +1508,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I28" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J28" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1517,7 +1517,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L28" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M28" s="10" t="str">
         <x:v>This is only based on manual subtitles; auto-captions are not used for the shortcut path.</x:v>
@@ -1590,7 +1590,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I30" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J30" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1599,7 +1599,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L30" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M30" s="10" t="str">
         <x:v>Style metadata on timing lines is ignored after the end timestamp.</x:v>
@@ -1631,7 +1631,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I31" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J31" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1640,7 +1640,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L31" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M31" s="10" t="str">
         <x:v>Malformed payloads return a parsing error.</x:v>
@@ -1754,7 +1754,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I34" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J34" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1763,7 +1763,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L34" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M34" s="10" t="str">
         <x:v>Repo instructions explicitly warn not to rely only on `which` when reasoning about this binary.</x:v>
@@ -1795,7 +1795,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I35" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J35" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1804,7 +1804,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L35" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M35" s="10" t="str">
         <x:v>Default-mode parsing surfaces these notices instead of hard-failing.</x:v>
@@ -1836,7 +1836,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I36" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J36" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1845,7 +1845,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L36" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M36" s="10" t="str">
         <x:v>Smoke tests verify the arguments written to a fake helper.</x:v>
@@ -1877,7 +1877,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I37" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J37" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1886,7 +1886,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L37" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M37" s="10" t="str">
         <x:v>lseend payloads may omit speaker_count and still parse successfully.</x:v>
@@ -1918,7 +1918,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I38" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J38" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1927,7 +1927,7 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L38" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M38" s="10" t="str">
         <x:v>This is a targeted resilience escape hatch, not a general suppress-all-errors rule.</x:v>
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>8</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: update feature tracker after ux fixes
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="Ra58635771d374f78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R35032fff9d914cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R2c4e63e59fa04e0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R23f18060f8d54e3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -498,7 +498,7 @@
         <x:v>Automated tests passed and the README now states that speaker-aware text is the default on-disk output.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="4" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="str">
         <x:v>FT-CLI-03</x:v>
       </x:c>
@@ -536,7 +536,7 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="M4" s="10" t="str">
-        <x:v>Smoke coverage already proved normal destination modes, and the parser now rejects `--output` followed by another flag instead of writing to a file literally named after that flag.</x:v>
+        <x:v>Smoke coverage already proved normal destination modes; the parser now rejects `--output` followed by another flag instead of writing to a file literally named after that flag; and slash-suffixed missing destinations such as `exports/` now resolve as directory intent using the default output filename.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1687,7 +1687,7 @@
         <x:v>Times, speed, and local-model markers are zeroed in the manual subtitle result; README now matches the narrower condition that this path only applies when diarization is inactive and `--local` is not set.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="66" hidden="0" customHeight="1">
+    <x:row r="33" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A33" s="11" t="str">
         <x:v>FT-REMOTE-09</x:v>
       </x:c>
@@ -1716,16 +1716,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="J33" s="12" t="str">
-        <x:v>None logged</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K33" s="12" t="str">
-        <x:v>Not needed</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L33" s="12" t="str">
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="M33" s="10" t="str">
-        <x:v>Remote alias smoke tests cover the forced-local flags, and a full run on 2026-07-01 against the README sample YouTube URL completed with `transcript_source = downloaded-audio-local-model`.</x:v>
+        <x:v>Remote alias smoke tests cover the forced-local flags; a full run on 2026-07-01 against the README sample YouTube URL completed with `transcript_source = downloaded-audio-local-model`; and release-only smoke tests now prove subtitle download and json3 parse failures fall back to downloaded audio instead of aborting.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="66" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh tracker after local pipeline fixes
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R2c4e63e59fa04e0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R23f18060f8d54e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R11c7e22f7a844e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rdb368b609ef2436a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1031,7 +1031,7 @@
         <x:v>Local pytest now skips this check when no wheel has been built, and after generating `dist-pypi/fscript-1.1.3-*.whl` the parity test passes end to end.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="17" ht="66" hidden="0" customHeight="1">
       <x:c r="A17" s="11" t="str">
         <x:v>FT-LP-01</x:v>
       </x:c>
@@ -1057,19 +1057,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I17" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J17" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K17" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L17" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M17" s="10" t="str">
-        <x:v>No checksum/version validation; a bad cached tarball is reused before failing.</x:v>
+        <x:v>Focused model tests now prove an existing incomplete custom model dir is repaired from a cached package; checksum/version validation is still absent, so a bad cached tarball is reused before failing.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1139,19 +1139,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I19" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J19" s="12" t="str">
-        <x:v>Edge-case risk</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K19" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L19" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M19" s="10" t="str">
-        <x:v>Zero-length audio would risk `inf`/`NaN` timing ratios.</x:v>
+        <x:v>Targeted transcribe tests now keep zero-length derived timing ratios finite instead of serializing non-finite values into the benchmark result; broader end-to-end coverage remains partial.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh tracker after renderer fixes
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R11c7e22f7a844e52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rdb368b609ef2436a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R67092fe3200e4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9c40a05e0ce14086"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -662,7 +662,7 @@
         <x:v>Verified by new unit and CLI smoke tests: invalid spaced values after `--speakers` or `--text` now error instead of becoming positional output paths.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="8" ht="66" hidden="0" customHeight="1">
       <x:c r="A8" s="11" t="str">
         <x:v>FT-CLI-07</x:v>
       </x:c>
@@ -691,19 +691,19 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="J8" s="12" t="str">
-        <x:v>Edge behavior only</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L8" s="12" t="str">
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="M8" s="10" t="str">
-        <x:v>If `segments` is absent, speaker output renders as an empty string.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Missing speaker labels intentionally omit any `UNKNOWN:` prefix, and speaker-aware output now errors clearly instead of silently rendering empty output when only plain transcript text is available without segment metadata.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
       <x:c r="A9" s="11" t="str">
         <x:v>FT-CLI-08</x:v>
       </x:c>
@@ -732,16 +732,16 @@
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="J9" s="12" t="str">
-        <x:v>Missing-segment gap</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L9" s="12" t="str">
         <x:v>Passed</x:v>
       </x:c>
       <x:c r="M9" s="10" t="str">
-        <x:v>Timestamped text with no segments renders empty output.</x:v>
+        <x:v>Plain and compact text still fall back to `result.text`; timestamped text now fails clearly instead of silently rendering empty output when only plain transcript text is available without segment metadata.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1959,19 +1959,19 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I39" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J39" s="12" t="str">
-        <x:v>Semantic mismatch only</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="K39" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="L39" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M39" s="10" t="str">
-        <x:v>Unlike the main Rust output path, missing speakers become the configured unknown label instead of silently omitting a prefix.</x:v>
+        <x:v>The helper now matches the main Rust output path by omitting a synthetic speaker prefix when labels are missing by default, while still allowing an explicit `--unknown-speaker-label` override.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh tracker after remote shortcut coverage
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R67092fe3200e4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R9c40a05e0ce14086"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R1ecf99ee424243e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R77dc245b703a4fbc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1523,7 +1523,7 @@
         <x:v>This is only based on manual subtitles; auto-captions are not used for the shortcut path.</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="29" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A29" s="11" t="str">
         <x:v>FT-REMOTE-05</x:v>
       </x:c>
@@ -1543,25 +1543,25 @@
         <x:v>src/remote.rs:54; src/remote.rs:233</x:v>
       </x:c>
       <x:c r="G29" s="12" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H29" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I29" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J29" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L29" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M29" s="10" t="str">
-        <x:v>Selection logic is implemented but not unit-tested directly.</x:v>
+        <x:v>Release-only CLI smoke tests now prove that manual subtitle shortcutting selects `json3` by default and prefers `vtt` when the chosen language exposes a VTT track.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1646,7 +1646,7 @@
         <x:v>Malformed payloads return a parsing error.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="66" hidden="0" customHeight="1">
+    <x:row r="32" ht="105.5999984741211" hidden="0" customHeight="1">
       <x:c r="A32" s="11" t="str">
         <x:v>FT-REMOTE-08</x:v>
       </x:c>
@@ -1666,25 +1666,25 @@
         <x:v>src/lib.rs:84; src/lib.rs:135; src/remote.rs:233</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H32" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I32" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J32" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L32" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M32" s="10" t="str">
-        <x:v>Times, speed, and local-model markers are zeroed in the manual subtitle result; README now matches the narrower condition that this path only applies when diarization is inactive and `--local` is not set.</x:v>
+        <x:v>Release-only CLI smoke tests now prove the manual subtitle shortcut path for both json3 and VTT tracks; the manual-subtitle benchmark result still zeroes timing and local-model markers, and the README matches the narrower condition that this path only applies when diarization is inactive and `--local` is not set.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="105.5999984741211" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh tracker after coverage updates
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R1ecf99ee424243e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R77dc245b703a4fbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R7dd2f6da13bf4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R15120ec0694d44e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -785,7 +785,7 @@
         <x:v>Missing-helper warnings are intentionally suppressed in text mode.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A11" s="11" t="str">
         <x:v>FT-CLI-10</x:v>
       </x:c>
@@ -805,28 +805,28 @@
         <x:v>src/types.rs:105; src/types.rs:124; src/output.rs:441; README.md:376</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I11" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J11" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L11" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M11" s="10" t="str">
-        <x:v>Tests assert some fields but do not lock the full schema.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>Unit coverage now asserts core JSON field names and values and proves optional `segments` and `speaker_diarization` fields are omitted when absent.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A12" s="11" t="str">
         <x:v>FT-CLI-11</x:v>
       </x:c>
@@ -846,25 +846,25 @@
         <x:v>src/output.rs:402; src/output.rs:420; src/output.rs:929; README.md:262</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I12" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J12" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L12" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M12" s="10" t="str">
-        <x:v>VTT with no valid cues becomes just `WEBVTT`; empty-SRT behavior is code-defined but lightly tested.</x:v>
+        <x:v>Unit coverage now directly proves SRT and VTT rendering, including speaker prefixes and skipping empty or non-positive segments; VTT with no valid cues still becomes just `WEBVTT`.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1195,7 +1195,7 @@
         <x:v>Sample rounding can shift exact chunk boundaries slightly.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="21" ht="66" hidden="0" customHeight="1">
       <x:c r="A21" s="11" t="str">
         <x:v>FT-LP-05</x:v>
       </x:c>
@@ -1221,7 +1221,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I21" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J21" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1230,13 +1230,13 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L21" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M21" s="10" t="str">
-        <x:v>Dedup depends on normalization that strips non-alphanumeric edges.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="52.79999923706055" hidden="0" customHeight="1">
+        <x:v>Unit coverage now directly exercises case-insensitive overlap dedup and the punctuation rule for one-word overlaps; dedup still depends on normalization that strips non-alphanumeric edges.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="66" hidden="0" customHeight="1">
       <x:c r="A22" s="11" t="str">
         <x:v>FT-LP-06</x:v>
       </x:c>
@@ -1262,7 +1262,7 @@
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I22" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J22" s="12" t="str">
         <x:v>None logged</x:v>
@@ -1271,10 +1271,10 @@
         <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L22" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M22" s="10" t="str">
-        <x:v>Only temporally overlapping segments are candidates for merge.</x:v>
+        <x:v>Unit coverage now directly exercises both fallback-segment creation when model segments are missing/invalid and overlap-based segment merging; only temporally overlapping segments are candidates for merge.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -1400,7 +1400,7 @@
         <x:v>Non-HTTP remote schemes are not supported.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="26" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A26" s="11" t="str">
         <x:v>FT-REMOTE-02</x:v>
       </x:c>
@@ -1420,25 +1420,25 @@
         <x:v>src/remote.rs:77; README.md:75</x:v>
       </x:c>
       <x:c r="G26" s="12" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I26" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J26" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K26" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L26" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M26" s="10" t="str">
-        <x:v>Important repo contract, currently untested in-code.</x:v>
+        <x:v>Release-only CLI smoke tests now prove the remote manual-subtitle shortcut still works when `yt-dlp` is absent from PATH but `uvx yt-dlp` is available.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>31</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
chore: refresh tracker after final coverage pass
</commit_message>
<xml_diff>
--- a/work/goals/feature-audit/feature-tracker.xlsx
+++ b/work/goals/feature-audit/feature-tracker.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R7dd2f6da13bf4d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R15120ec0694d44e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Features" sheetId="1" r:id="R71c18e174e5d4000"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rd6cd7f5634fe43c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1072,7 +1072,7 @@
         <x:v>Focused model tests now prove an existing incomplete custom model dir is repaired from a cached package; checksum/version validation is still absent, so a bad cached tarball is reused before failing.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="18" ht="66" hidden="0" customHeight="1">
       <x:c r="A18" s="11" t="str">
         <x:v>FT-LP-02</x:v>
       </x:c>
@@ -1092,25 +1092,25 @@
         <x:v>src/audio.rs:35; src/audio.rs:43; src/types.rs:71</x:v>
       </x:c>
       <x:c r="G18" s="12" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I18" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J18" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K18" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L18" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M18" s="10" t="str">
-        <x:v>Missing `ffprobe` or `ffmpeg` hard-fails the run.</x:v>
+        <x:v>Unit coverage now proves supported 16 kHz mono PCM16 audio is reused without running ffmpeg and unsupported audio is normalized into a temp WAV; missing `ffprobe` or `ffmpeg` still hard-fails the run.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="52.79999923706055" hidden="0" customHeight="1">
@@ -1318,7 +1318,7 @@
         <x:v>Kept as pipeline behavior because it changes the post-ASR data shape.</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="24" ht="66" hidden="0" customHeight="1">
       <x:c r="A24" s="11" t="str">
         <x:v>FT-LP-08</x:v>
       </x:c>
@@ -1338,25 +1338,25 @@
         <x:v>src/transcribe.rs:211; src/progress.rs:7; src/progress.rs:29</x:v>
       </x:c>
       <x:c r="G24" s="12" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="H24" s="12" t="str">
         <x:v>Audited</x:v>
       </x:c>
       <x:c r="I24" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J24" s="12" t="str">
-        <x:v>Coverage gap</x:v>
+        <x:v>None logged</x:v>
       </x:c>
       <x:c r="K24" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Not needed</x:v>
       </x:c>
       <x:c r="L24" s="12" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="M24" s="10" t="str">
-        <x:v>Formatting is tested; thread and join behavior are not.</x:v>
+        <x:v>Unit coverage now proves interactive and non-interactive reporter lifecycles, including the background-thread join path, and locks the coarse non-TTY status messages alongside the existing formatting tests.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2045,7 +2045,7 @@
       </x:c>
       <x:c r="E5" s="23" t="n">
         <x:f>COUNTIF(Features!$I$2:$I$39,"&lt;&gt;Not started")</x:f>
-        <x:v>36</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -2060,7 +2060,7 @@
       </x:c>
       <x:c r="E6" s="23" t="n">
         <x:f>COUNTIF(Features!$J$2:$J$39,"&lt;&gt;None logged")</x:f>
-        <x:v>15</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">

</xml_diff>